<commit_message>
Update: Vijaywada-April-2026 by admin
</commit_message>
<xml_diff>
--- a/Vijaywada-April-2026.xlsx
+++ b/Vijaywada-April-2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Accounts\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D5A7E57F-69E3-4091-81DC-8DF3816C6EA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7323A5A-634A-4377-B00B-C334BACD0199}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{87F3F403-B311-4F47-89B4-47D1FE63D0D3}"/>
   </bookViews>
@@ -41,9 +41,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="31">
   <si>
-    <t>Vijayawada</t>
-  </si>
-  <si>
     <t>April</t>
   </si>
   <si>
@@ -132,6 +129,9 @@
   </si>
   <si>
     <t>CRYSTA</t>
+  </si>
+  <si>
+    <t>Vijaywada</t>
   </si>
 </sst>
 </file>
@@ -591,82 +591,82 @@
   <sheetData>
     <row r="1" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>28</v>
-      </c>
-      <c r="Z1" s="1" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.3">
@@ -674,19 +674,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D2" s="3">
         <v>2026</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G2" s="4">
         <v>44278</v>
@@ -754,19 +754,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3" s="3">
         <v>2026</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G3" s="4">
         <v>44461</v>

</xml_diff>